<commit_message>
Erfan/water sales split (#70)
</commit_message>
<xml_diff>
--- a/src/Datiss.Budget.Web/wwwroot/excel/WasteInstallFeeImport.xlsx
+++ b/src/Datiss.Budget.Web/wwwroot/excel/WasteInstallFeeImport.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="24527"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="24701"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\FinalDatiss\Datiss\datiss.budget\src\Datiss.Budget.Web\wwwroot\excel\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Budget.Datiss\datiss.budget\src\Datiss.Budget.Web\wwwroot\excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ACD2F1AA-BD82-4C9B-AB25-E7487877DC7F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1B419781-269F-4342-8CA1-295A47A5B3A1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="12852" yWindow="0" windowWidth="10188" windowHeight="12360" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="8544" yWindow="0" windowWidth="10188" windowHeight="12360" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -27,16 +27,16 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4" uniqueCount="4">
   <si>
-    <t>Column1</t>
+    <t>سال</t>
   </si>
   <si>
-    <t>Column2</t>
+    <t>سازمان</t>
   </si>
   <si>
-    <t>Column3</t>
+    <t>کاربری</t>
   </si>
   <si>
-    <t>Column4</t>
+    <t>قیمت</t>
   </si>
 </sst>
 </file>
@@ -73,13 +73,20 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
+  <dxfs count="1">
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
@@ -93,13 +100,13 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Table1" displayName="Table1" ref="A1:D3" totalsRowShown="0">
-  <autoFilter ref="A1:D3" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Table1" displayName="Table1" ref="A1:D2" insertRow="1" totalsRowShown="0" headerRowDxfId="0">
+  <autoFilter ref="A1:D2" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
   <tableColumns count="4">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="Column1"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="Column2"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="Column3"/>
-    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="Column4"/>
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="سال"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="سازمان"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="کاربری"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="قیمت"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -368,52 +375,24 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D3"/>
+  <dimension ref="A1:D1"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="4" width="11" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A1" t="s">
+    <row r="1" spans="1:4" s="1" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
-      </c>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A2">
-        <v>1</v>
-      </c>
-      <c r="B2">
-        <v>1</v>
-      </c>
-      <c r="C2">
-        <v>1</v>
-      </c>
-      <c r="D2">
-        <v>890000</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A3">
-        <v>1</v>
-      </c>
-      <c r="B3">
-        <v>2</v>
-      </c>
-      <c r="C3">
-        <v>2</v>
-      </c>
-      <c r="D3">
-        <v>90000</v>
       </c>
     </row>
   </sheetData>

</xml_diff>